<commit_message>
F: feedback from xialong (14:40) appllied
</commit_message>
<xml_diff>
--- a/tests/test_plan_v1.xlsx
+++ b/tests/test_plan_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/minhakim/Project/glucolink-a2/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9DF58C80-7593-154E-851C-D19ACD047483}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC32D8F0-D8D3-994C-91AD-BA9BF49FD26A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13680" yWindow="680" windowWidth="17280" windowHeight="19940" xr2:uid="{38C2F623-CE48-954F-9147-651889642CF7}"/>
+    <workbookView xWindow="12980" yWindow="680" windowWidth="21580" windowHeight="19940" activeTab="1" xr2:uid="{38C2F623-CE48-954F-9147-651889642CF7}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Plan v1.1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="296">
   <si>
     <t>Test ID</t>
   </si>
@@ -739,11 +739,6 @@
     <t>After run 2: tests = passed (all rows of audit.test_result), failed 0; raw_runs 2; all layer counts identical to run 1</t>
   </si>
   <si>
-    <t>SELECT count(*) AS n_rows
-  FROM reporting.vw_uc4_care_path_breaks
-  WHERE detail LIKE '%OBS-0031%' OR detail LIKE '%MSG-0032%' OR patient_id = 'GL-0009';</t>
-  </si>
-  <si>
     <t>n_rows 0</t>
   </si>
   <si>
@@ -986,15 +981,9 @@
     <t>Y</t>
   </si>
   <si>
-    <t>N</t>
-  </si>
-  <si>
     <t>2026-10-07_C_part2_counts.png</t>
   </si>
   <si>
-    <t xml:space="preserve"> 2026-10-07_D_patient_record.png</t>
-  </si>
-  <si>
     <t>2026-10-07_D_identity_counts.png</t>
   </si>
   <si>
@@ -1013,16 +1002,10 @@
     <t>2026-10-08_F_dashboard_tool.png</t>
   </si>
   <si>
-    <t xml:space="preserve"> 2026-10-09_E_fact_counts.png</t>
-  </si>
-  <si>
     <t>2026-10-09_D_vw_uc2.png</t>
   </si>
   <si>
     <t>2026-10-09_E_vw_uc1_uc3.png</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 2026-10-10_D_vw_uc4.png</t>
   </si>
   <si>
     <t>2026-10-10_F_test_results.png</t>
@@ -1073,13 +1056,33 @@
     <t>NEGATIVE - a high result followed by a qualifying review visit within 90 days (P13: 60.0 on 2026-04-10, review 2026-05-02) and a patient whose latest result is below the threshold</t>
   </si>
   <si>
+    <t>n_rows 48 | persons 18 | known_system 48 (plus: no statement in sql/04 or sql/05 reads audit.identity_truth - comments don't count)</t>
+  </si>
+  <si>
+    <t>SELECT count(*) AS n_rows FROM reporting.vw_uc1_care_gaps WHERE patient_id IN ('GL-0013','GL-0009');</t>
+  </si>
+  <si>
     <t>SELECT count(*) AS n_rows
   FROM reporting.vw_uc4_care_path_breaks
-  WHERE detail LIKE '%OBS-0031%' OR detail LIKE '%MSG-0032%'
-     OR patient_id = 'GL-0015' OR patient_id = 'GL-0009';</t>
-  </si>
-  <si>
-    <t>n_rows 48 | persons 18 | known_system 48 (plus: no statement in sql/04 or sql/05 reads audit.identity_truth - comments don't count)</t>
+  WHERE detail LIKE '%OBS-0031%' OR detail LIKE '%MSG-0032%' OR patient_id = 'GL-0009' OR patient_id = 'GL-0015';</t>
+  </si>
+  <si>
+    <t>identity_truth split and flags missing;</t>
+  </si>
+  <si>
+    <t>no-Medicare and sex-type screenshots missing;</t>
+  </si>
+  <si>
+    <t>no SQL visible</t>
+  </si>
+  <si>
+    <t>2026-10-07_D_patient_record.png</t>
+  </si>
+  <si>
+    <t>2026-10-09_E_fact_counts.png</t>
+  </si>
+  <si>
+    <t>2026-10-10_D_vw_uc4.png</t>
   </si>
 </sst>
 </file>
@@ -1225,12 +1228,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1245,62 +1242,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -1353,11 +1306,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1718,13 +1671,13 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>97</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="51" x14ac:dyDescent="0.2">
@@ -1747,7 +1700,7 @@
         <v>182</v>
       </c>
       <c r="G2" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="68" x14ac:dyDescent="0.2">
@@ -1770,7 +1723,7 @@
         <v>183</v>
       </c>
       <c r="G3" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="68" x14ac:dyDescent="0.2">
@@ -1793,7 +1746,7 @@
         <v>184</v>
       </c>
       <c r="G4" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="68" x14ac:dyDescent="0.2">
@@ -1810,13 +1763,13 @@
         <v>70</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>185</v>
       </c>
       <c r="G5" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="238" x14ac:dyDescent="0.2">
@@ -1830,7 +1783,7 @@
         <v>42</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>186</v>
@@ -1839,7 +1792,7 @@
         <v>187</v>
       </c>
       <c r="G6" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="85" x14ac:dyDescent="0.2">
@@ -1862,7 +1815,7 @@
         <v>107</v>
       </c>
       <c r="G7" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="85" x14ac:dyDescent="0.2">
@@ -1885,7 +1838,7 @@
         <v>106</v>
       </c>
       <c r="G8" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="51" x14ac:dyDescent="0.2">
@@ -1908,7 +1861,7 @@
         <v>188</v>
       </c>
       <c r="G9" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="34" x14ac:dyDescent="0.2">
@@ -1931,7 +1884,7 @@
         <v>111</v>
       </c>
       <c r="G10" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="68" x14ac:dyDescent="0.2">
@@ -1954,7 +1907,7 @@
         <v>115</v>
       </c>
       <c r="G11" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="68" x14ac:dyDescent="0.2">
@@ -1977,7 +1930,7 @@
         <v>140</v>
       </c>
       <c r="G12" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="51" x14ac:dyDescent="0.2">
@@ -2000,7 +1953,7 @@
         <v>74</v>
       </c>
       <c r="G13" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="34" x14ac:dyDescent="0.2">
@@ -2023,7 +1976,7 @@
         <v>77</v>
       </c>
       <c r="G14" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="102" x14ac:dyDescent="0.2">
@@ -2040,13 +1993,13 @@
         <v>165</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="G15" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="85" x14ac:dyDescent="0.2">
@@ -2069,7 +2022,7 @@
         <v>154</v>
       </c>
       <c r="G16" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="85" x14ac:dyDescent="0.2">
@@ -2092,7 +2045,7 @@
         <v>153</v>
       </c>
       <c r="G17" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="34" x14ac:dyDescent="0.2">
@@ -2115,7 +2068,7 @@
         <v>79</v>
       </c>
       <c r="G18" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="68" x14ac:dyDescent="0.2">
@@ -2138,7 +2091,7 @@
         <v>159</v>
       </c>
       <c r="G19" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="51" x14ac:dyDescent="0.2">
@@ -2161,7 +2114,7 @@
         <v>81</v>
       </c>
       <c r="G20" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="51" x14ac:dyDescent="0.2">
@@ -2184,7 +2137,7 @@
         <v>83</v>
       </c>
       <c r="G21" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="68" x14ac:dyDescent="0.2">
@@ -2207,7 +2160,7 @@
         <v>170</v>
       </c>
       <c r="G22" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="68" x14ac:dyDescent="0.2">
@@ -2230,7 +2183,7 @@
         <v>175</v>
       </c>
       <c r="G23" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="51" x14ac:dyDescent="0.2">
@@ -2253,7 +2206,7 @@
         <v>178</v>
       </c>
       <c r="G24" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="51" x14ac:dyDescent="0.2">
@@ -2276,7 +2229,7 @@
         <v>181</v>
       </c>
       <c r="G25" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="68" x14ac:dyDescent="0.2">
@@ -2299,7 +2252,7 @@
         <v>164</v>
       </c>
       <c r="G26" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="404" x14ac:dyDescent="0.2">
@@ -2322,7 +2275,7 @@
         <v>168</v>
       </c>
       <c r="G27" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="68" x14ac:dyDescent="0.2">
@@ -2345,10 +2298,10 @@
         <v>189</v>
       </c>
       <c r="G28" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="119" x14ac:dyDescent="0.2">
       <c r="A29" s="6" t="s">
         <v>23</v>
       </c>
@@ -2368,7 +2321,7 @@
         <v>121</v>
       </c>
       <c r="G29" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="34" x14ac:dyDescent="0.2">
@@ -2388,10 +2341,10 @@
         <v>85</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="G30" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="68" x14ac:dyDescent="0.2">
@@ -2402,19 +2355,19 @@
         <v>37</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G31" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="51" x14ac:dyDescent="0.2">
@@ -2437,10 +2390,10 @@
         <v>87</v>
       </c>
       <c r="G32" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="153" x14ac:dyDescent="0.2">
       <c r="A33" s="6" t="s">
         <v>25</v>
       </c>
@@ -2460,7 +2413,7 @@
         <v>126</v>
       </c>
       <c r="G33" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="51" x14ac:dyDescent="0.2">
@@ -2483,7 +2436,7 @@
         <v>98</v>
       </c>
       <c r="G34" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="68" x14ac:dyDescent="0.2">
@@ -2506,7 +2459,7 @@
         <v>191</v>
       </c>
       <c r="G35" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="51" x14ac:dyDescent="0.2">
@@ -2529,10 +2482,10 @@
         <v>90</v>
       </c>
       <c r="G36" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="102" x14ac:dyDescent="0.2">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="204" x14ac:dyDescent="0.2">
       <c r="A37" s="6" t="s">
         <v>28</v>
       </c>
@@ -2552,7 +2505,7 @@
         <v>132</v>
       </c>
       <c r="G37" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="51" x14ac:dyDescent="0.2">
@@ -2575,7 +2528,7 @@
         <v>99</v>
       </c>
       <c r="G38" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="85" x14ac:dyDescent="0.2">
@@ -2586,19 +2539,19 @@
         <v>39</v>
       </c>
       <c r="C39" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="D39" s="2" t="s">
+      <c r="E39" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="E39" s="4" t="s">
+      <c r="F39" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="F39" s="2" t="s">
-        <v>200</v>
-      </c>
       <c r="G39" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="51" x14ac:dyDescent="0.2">
@@ -2621,10 +2574,10 @@
         <v>144</v>
       </c>
       <c r="G40" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A41" s="6" t="s">
         <v>30</v>
       </c>
@@ -2644,7 +2597,7 @@
         <v>135</v>
       </c>
       <c r="G41" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="51" x14ac:dyDescent="0.2">
@@ -2661,13 +2614,13 @@
         <v>63</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>193</v>
+        <v>289</v>
       </c>
       <c r="G42" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="102" x14ac:dyDescent="0.2">
@@ -2686,11 +2639,11 @@
       <c r="E43" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="F43" s="21" t="s">
-        <v>286</v>
+      <c r="F43" s="19" t="s">
+        <v>281</v>
       </c>
       <c r="G43" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="85" x14ac:dyDescent="0.2">
@@ -2709,11 +2662,11 @@
       <c r="E44" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="F44" s="21" t="s">
-        <v>287</v>
+      <c r="F44" s="19" t="s">
+        <v>282</v>
       </c>
       <c r="G44" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
@@ -2730,40 +2683,20 @@
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="G2:G1048576">
-    <cfRule type="cellIs" dxfId="9" priority="6" operator="equal">
-      <formula>"Blocked"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="7" operator="equal">
-      <formula>"Fail"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="8" operator="equal">
-      <formula>"Pass"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G7">
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
+  <conditionalFormatting sqref="G2:G44">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
       <formula>"Not run"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G8">
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
-      <formula>"Not run"</formula>
+  <conditionalFormatting sqref="G2:G1048576">
+    <cfRule type="cellIs" dxfId="4" priority="6" operator="equal">
+      <formula>"Blocked"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G9">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
-      <formula>"Not run"</formula>
+    <cfRule type="cellIs" dxfId="3" priority="7" operator="equal">
+      <formula>"Fail"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G11:G44">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
-      <formula>"Not run"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G10">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
-      <formula>"Not run"</formula>
+    <cfRule type="cellIs" dxfId="2" priority="8" operator="equal">
+      <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -2783,445 +2716,458 @@
     <col min="1" max="1" width="10.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="5.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="29.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="41.5" style="16" customWidth="1"/>
+    <col min="5" max="5" width="41.5" style="14" customWidth="1"/>
     <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22" style="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="21" t="s">
+        <v>209</v>
+      </c>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="20"/>
+      <c r="L2" s="20"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3" s="20" t="s">
         <v>210</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A2" s="15" t="s">
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="20"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A4" s="20" t="s">
+        <v>211</v>
+      </c>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="20"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A5" s="20" t="s">
         <v>213</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" s="15" t="s">
-        <v>211</v>
-      </c>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A4" s="15" t="s">
-        <v>212</v>
-      </c>
-      <c r="B4" s="15"/>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15"/>
-      <c r="I4" s="15"/>
-      <c r="J4" s="15"/>
-      <c r="K4" s="15"/>
-      <c r="L4" s="15"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5" s="15" t="s">
-        <v>214</v>
-      </c>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="20"/>
     </row>
     <row r="9" spans="1:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="16" t="s">
+        <v>201</v>
+      </c>
+      <c r="B9" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="C9" s="16" t="s">
         <v>203</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="D9" s="16" t="s">
         <v>204</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="E9" s="17" t="s">
         <v>205</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="F9" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="G9" s="16" t="s">
         <v>207</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="H9" s="17" t="s">
         <v>208</v>
       </c>
-      <c r="H9" s="18" t="s">
-        <v>209</v>
-      </c>
     </row>
     <row r="10" spans="1:12" ht="34" x14ac:dyDescent="0.2">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="14" t="s">
+        <v>216</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="C10" t="s">
+        <v>279</v>
+      </c>
+      <c r="D10" t="s">
+        <v>236</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>249</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="G10" s="18">
+        <v>46303</v>
+      </c>
+      <c r="H10" s="14" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="A11" s="14" t="s">
+        <v>216</v>
+      </c>
+      <c r="B11" s="14" t="s">
         <v>217</v>
       </c>
-      <c r="B10" s="16" t="s">
-        <v>216</v>
-      </c>
-      <c r="C10" t="s">
-        <v>284</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="C11" t="s">
+        <v>223</v>
+      </c>
+      <c r="D11" t="s">
+        <v>248</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>250</v>
+      </c>
+      <c r="F11" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="G11" s="18">
+        <v>46303</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="A12" s="14" t="s">
         <v>237</v>
       </c>
-      <c r="E10" s="16" t="s">
-        <v>250</v>
-      </c>
-      <c r="F10" s="16" t="s">
+      <c r="B12" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="C12" t="s">
+        <v>222</v>
+      </c>
+      <c r="D12" t="s">
         <v>267</v>
       </c>
-      <c r="G10" s="20">
+      <c r="E12" s="14" t="s">
+        <v>251</v>
+      </c>
+      <c r="F12" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="G12" s="18">
         <v>46303</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" ht="34" x14ac:dyDescent="0.2">
-      <c r="A11" s="16" t="s">
+      <c r="H12" s="14" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="A13" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>218</v>
+      </c>
+      <c r="C13" t="s">
+        <v>224</v>
+      </c>
+      <c r="D13" t="s">
+        <v>293</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>252</v>
+      </c>
+      <c r="F13" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="G13" s="18">
+        <v>46302</v>
+      </c>
+      <c r="H13" s="14" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="A14" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>218</v>
+      </c>
+      <c r="C14" t="s">
+        <v>225</v>
+      </c>
+      <c r="D14" t="s">
+        <v>268</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>253</v>
+      </c>
+      <c r="F14" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="G14" s="18">
+        <v>46302</v>
+      </c>
+      <c r="H14" s="14" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="A15" s="14" t="s">
+        <v>238</v>
+      </c>
+      <c r="B15" s="14" t="s">
         <v>217</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="C15" t="s">
+        <v>226</v>
+      </c>
+      <c r="D15" t="s">
+        <v>269</v>
+      </c>
+      <c r="E15" s="14" t="s">
+        <v>254</v>
+      </c>
+      <c r="F15" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="G15" s="18">
+        <v>46303</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="A16" s="14" t="s">
+        <v>239</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="C16" t="s">
+        <v>227</v>
+      </c>
+      <c r="D16" t="s">
+        <v>270</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>255</v>
+      </c>
+      <c r="F16" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="G16" s="18">
+        <v>46303</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="68" x14ac:dyDescent="0.2">
+      <c r="A17" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="B17" s="14" t="s">
         <v>218</v>
       </c>
-      <c r="C11" t="s">
-        <v>224</v>
-      </c>
-      <c r="D11" t="s">
-        <v>249</v>
-      </c>
-      <c r="E11" s="16" t="s">
-        <v>251</v>
-      </c>
-      <c r="F11" s="16" t="s">
-        <v>267</v>
-      </c>
-      <c r="G11" s="20">
-        <v>46303</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="34" x14ac:dyDescent="0.2">
-      <c r="A12" s="16" t="s">
-        <v>238</v>
-      </c>
-      <c r="B12" s="16" t="s">
-        <v>216</v>
-      </c>
-      <c r="C12" t="s">
-        <v>223</v>
-      </c>
-      <c r="D12" t="s">
-        <v>269</v>
-      </c>
-      <c r="E12" s="16" t="s">
-        <v>252</v>
-      </c>
-      <c r="F12" s="16" t="s">
-        <v>267</v>
-      </c>
-      <c r="G12" s="20">
-        <v>46303</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="34" x14ac:dyDescent="0.2">
-      <c r="A13" s="16" t="s">
-        <v>238</v>
-      </c>
-      <c r="B13" s="16" t="s">
+      <c r="C17" t="s">
+        <v>228</v>
+      </c>
+      <c r="D17" t="s">
+        <v>271</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A18" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="B18" s="14" t="s">
         <v>219</v>
       </c>
-      <c r="C13" t="s">
-        <v>225</v>
-      </c>
-      <c r="D13" t="s">
-        <v>270</v>
-      </c>
-      <c r="E13" s="16" t="s">
-        <v>253</v>
-      </c>
-      <c r="F13" s="16" t="s">
-        <v>268</v>
-      </c>
-      <c r="G13" s="20">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="34" x14ac:dyDescent="0.2">
-      <c r="A14" s="16" t="s">
-        <v>238</v>
-      </c>
-      <c r="B14" s="16" t="s">
+      <c r="C18" t="s">
+        <v>229</v>
+      </c>
+      <c r="D18" t="s">
+        <v>272</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A19" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="C19" t="s">
+        <v>230</v>
+      </c>
+      <c r="D19" t="s">
+        <v>273</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A20" s="14" t="s">
+        <v>241</v>
+      </c>
+      <c r="B20" s="14" t="s">
         <v>219</v>
       </c>
-      <c r="C14" t="s">
-        <v>226</v>
-      </c>
-      <c r="D14" t="s">
-        <v>271</v>
-      </c>
-      <c r="E14" s="16" t="s">
-        <v>254</v>
-      </c>
-      <c r="F14" s="16" t="s">
-        <v>268</v>
-      </c>
-      <c r="G14" s="20">
-        <v>46302</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="34" x14ac:dyDescent="0.2">
-      <c r="A15" s="16" t="s">
-        <v>239</v>
-      </c>
-      <c r="B15" s="16" t="s">
+      <c r="C20" t="s">
+        <v>231</v>
+      </c>
+      <c r="D20" t="s">
+        <v>294</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A21" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="B21" s="14" t="s">
         <v>218</v>
       </c>
-      <c r="C15" t="s">
-        <v>227</v>
-      </c>
-      <c r="D15" t="s">
-        <v>272</v>
-      </c>
-      <c r="E15" s="16" t="s">
-        <v>255</v>
-      </c>
-      <c r="F15" s="16" t="s">
-        <v>267</v>
-      </c>
-      <c r="G15" s="20">
-        <v>46303</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="34" x14ac:dyDescent="0.2">
-      <c r="A16" s="16" t="s">
-        <v>240</v>
-      </c>
-      <c r="B16" s="16" t="s">
-        <v>216</v>
-      </c>
-      <c r="C16" t="s">
-        <v>228</v>
-      </c>
-      <c r="D16" t="s">
-        <v>273</v>
-      </c>
-      <c r="E16" s="16" t="s">
-        <v>256</v>
-      </c>
-      <c r="F16" s="16" t="s">
-        <v>267</v>
-      </c>
-      <c r="G16" s="20">
-        <v>46303</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="68" x14ac:dyDescent="0.2">
-      <c r="A17" s="16" t="s">
-        <v>241</v>
-      </c>
-      <c r="B17" s="16" t="s">
+      <c r="C21" t="s">
+        <v>232</v>
+      </c>
+      <c r="D21" t="s">
+        <v>274</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A22" s="14" t="s">
+        <v>244</v>
+      </c>
+      <c r="B22" s="14" t="s">
         <v>219</v>
       </c>
-      <c r="C17" t="s">
-        <v>229</v>
-      </c>
-      <c r="D17" t="s">
-        <v>274</v>
-      </c>
-      <c r="E17" s="16" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A18" s="16" t="s">
-        <v>241</v>
-      </c>
-      <c r="B18" s="16" t="s">
+      <c r="C22" t="s">
+        <v>233</v>
+      </c>
+      <c r="D22" t="s">
+        <v>275</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A23" s="15" t="s">
+        <v>243</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>218</v>
+      </c>
+      <c r="C23" t="s">
+        <v>232</v>
+      </c>
+      <c r="D23" t="s">
+        <v>295</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A24" s="15" t="s">
+        <v>247</v>
+      </c>
+      <c r="B24" s="14" t="s">
         <v>220</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C24" t="s">
+        <v>234</v>
+      </c>
+      <c r="D24" t="s">
+        <v>276</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A25" s="14" t="s">
+        <v>245</v>
+      </c>
+      <c r="B25" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="C25" t="s">
         <v>230</v>
       </c>
-      <c r="D18" t="s">
-        <v>275</v>
-      </c>
-      <c r="E18" s="16" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A19" s="16" t="s">
-        <v>241</v>
-      </c>
-      <c r="B19" s="16" t="s">
+      <c r="D25" t="s">
+        <v>277</v>
+      </c>
+      <c r="E25" s="14" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A26" s="14" t="s">
+        <v>246</v>
+      </c>
+      <c r="B26" s="14" t="s">
         <v>221</v>
       </c>
-      <c r="C19" t="s">
-        <v>231</v>
-      </c>
-      <c r="D19" t="s">
-        <v>276</v>
-      </c>
-      <c r="E19" s="16" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A20" s="16" t="s">
-        <v>242</v>
-      </c>
-      <c r="B20" s="16" t="s">
-        <v>220</v>
-      </c>
-      <c r="C20" t="s">
-        <v>232</v>
-      </c>
-      <c r="D20" t="s">
-        <v>277</v>
-      </c>
-      <c r="E20" s="16" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A21" s="16" t="s">
-        <v>243</v>
-      </c>
-      <c r="B21" s="16" t="s">
-        <v>219</v>
-      </c>
-      <c r="C21" t="s">
-        <v>233</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="C26" t="s">
+        <v>235</v>
+      </c>
+      <c r="D26" t="s">
         <v>278</v>
       </c>
-      <c r="E21" s="16" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A22" s="16" t="s">
-        <v>245</v>
-      </c>
-      <c r="B22" s="16" t="s">
-        <v>220</v>
-      </c>
-      <c r="C22" t="s">
-        <v>234</v>
-      </c>
-      <c r="D22" t="s">
-        <v>279</v>
-      </c>
-      <c r="E22" s="16" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A23" s="17" t="s">
-        <v>244</v>
-      </c>
-      <c r="B23" s="16" t="s">
-        <v>219</v>
-      </c>
-      <c r="C23" t="s">
-        <v>233</v>
-      </c>
-      <c r="D23" t="s">
-        <v>280</v>
-      </c>
-      <c r="E23" s="16" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A24" s="17" t="s">
-        <v>248</v>
-      </c>
-      <c r="B24" s="16" t="s">
-        <v>221</v>
-      </c>
-      <c r="C24" t="s">
-        <v>235</v>
-      </c>
-      <c r="D24" t="s">
-        <v>281</v>
-      </c>
-      <c r="E24" s="16" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A25" s="16" t="s">
-        <v>246</v>
-      </c>
-      <c r="B25" s="16" t="s">
-        <v>221</v>
-      </c>
-      <c r="C25" t="s">
-        <v>231</v>
-      </c>
-      <c r="D25" t="s">
-        <v>282</v>
-      </c>
-      <c r="E25" s="16" t="s">
+      <c r="E26" s="14" t="s">
         <v>265</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A26" s="16" t="s">
-        <v>247</v>
-      </c>
-      <c r="B26" s="16" t="s">
-        <v>222</v>
-      </c>
-      <c r="C26" t="s">
-        <v>236</v>
-      </c>
-      <c r="D26" t="s">
-        <v>283</v>
-      </c>
-      <c r="E26" s="16" t="s">
-        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -3233,10 +3179,10 @@
     <mergeCell ref="A1:L1"/>
   </mergeCells>
   <conditionalFormatting sqref="F10:F26">
-    <cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
F/test plan fix (#12)
* feat: excel updated

* f: dashboard options updated - add our decision, our chart plan

* feat: vw_uc2 updated in UC2

* feat: vw_uc2 evidence added

* feat: 09_tests.sql added

* feat: video outline
</commit_message>
<xml_diff>
--- a/tests/test_plan_v1.xlsx
+++ b/tests/test_plan_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/minhakim/Project/glucolink-a2/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC32D8F0-D8D3-994C-91AD-BA9BF49FD26A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A926E115-A6EB-CE42-831D-D7A54EC85F33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12980" yWindow="680" windowWidth="21580" windowHeight="19940" activeTab="1" xr2:uid="{38C2F623-CE48-954F-9147-651889642CF7}"/>
+    <workbookView xWindow="12980" yWindow="680" windowWidth="21580" windowHeight="19940" xr2:uid="{38C2F623-CE48-954F-9147-651889642CF7}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Plan v1.1" sheetId="1" r:id="rId1"/>

</xml_diff>